<commit_message>
Remove mesh animation from landing page
</commit_message>
<xml_diff>
--- a/assets/pricing_models/B.xlsx
+++ b/assets/pricing_models/B.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="7">
   <si>
     <t>B</t>
   </si>
@@ -30,6 +30,9 @@
   </si>
   <si>
     <t>المقاس</t>
+  </si>
+  <si>
+    <t>------</t>
   </si>
 </sst>
 </file>
@@ -198,53 +201,53 @@
         <color rgb="1800AD"/>
       </top>
       <bottom style="medium">
-        <color rgb="000000"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thick"/>
+        <color rgb="545454"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium"/>
       <top style="thick">
         <color rgb="1800AD"/>
       </top>
       <bottom style="medium">
-        <color rgb="000000"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="1800AD"/>
+        <color rgb="545454"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="545454"/>
       </left>
       <top style="thick">
         <color rgb="1800AD"/>
       </top>
       <bottom style="medium">
-        <color rgb="000000"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="1800AD"/>
-      </left>
-      <right style="thick"/>
+        <color rgb="545454"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="545454"/>
+      </left>
+      <right style="medium"/>
       <top style="thick">
         <color rgb="1800AD"/>
       </top>
       <bottom style="medium">
-        <color rgb="000000"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="1800AD"/>
-      </left>
-      <right style="thick">
-        <color rgb="1800AD"/>
+        <color rgb="545454"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="545454"/>
+      </left>
+      <right style="medium">
+        <color rgb="545454"/>
       </right>
       <top style="thick">
         <color rgb="1800AD"/>
       </top>
       <bottom style="medium">
-        <color rgb="000000"/>
+        <color rgb="545454"/>
       </bottom>
     </border>
     <border>
@@ -252,64 +255,64 @@
     </border>
     <border>
       <top style="medium">
-        <color rgb="000000"/>
+        <color rgb="545454"/>
       </top>
     </border>
     <border>
       <top style="medium">
-        <color rgb="000000"/>
+        <color rgb="545454"/>
       </top>
       <bottom style="thick"/>
     </border>
     <border>
       <top style="medium">
-        <color rgb="000000"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="1800AD"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thick"/>
+        <color rgb="545454"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="1800AD"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium"/>
       <top style="medium">
-        <color rgb="000000"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="1800AD"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="1800AD"/>
+        <color rgb="545454"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="1800AD"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="545454"/>
       </left>
       <top style="medium">
-        <color rgb="000000"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="1800AD"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="1800AD"/>
-      </left>
-      <right style="thick"/>
+        <color rgb="545454"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="1800AD"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="545454"/>
+      </left>
+      <right style="medium"/>
       <top style="medium">
-        <color rgb="000000"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="1800AD"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="1800AD"/>
-      </left>
-      <right style="thick">
-        <color rgb="1800AD"/>
+        <color rgb="545454"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="1800AD"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="545454"/>
+      </left>
+      <right style="medium">
+        <color rgb="545454"/>
       </right>
       <top style="medium">
-        <color rgb="000000"/>
+        <color rgb="545454"/>
       </top>
       <bottom style="thick">
         <color rgb="1800AD"/>
@@ -319,7 +322,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
       <alignment wrapText="true" horizontal="center"/>
@@ -334,12 +337,6 @@
       <alignment readingOrder="2" wrapText="true" horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="24" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
-      <alignment readingOrder="2" wrapText="true" horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true" applyNumberFormat="true">
-      <alignment readingOrder="2" wrapText="true" horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="6" borderId="24" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true" applyNumberFormat="true">
       <alignment readingOrder="2" wrapText="true" horizontal="center"/>
     </xf>
   </cellXfs>
@@ -388,7 +385,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="33.0" baseColWidth="16" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="16.5" customWidth="true"/>
@@ -421,121 +418,308 @@
       </c>
     </row>
     <row r="3" ht="54.0" customHeight="true">
-      <c r="A3" s="6" t="n">
-        <v>365.0</v>
-      </c>
-      <c r="B3" s="6" t="n">
-        <v>580.0</v>
-      </c>
-      <c r="C3" s="6" t="n">
-        <v>505.0</v>
-      </c>
-      <c r="D3" s="6" t="n">
-        <v>450.0</v>
+      <c r="A3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>230.0</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>205.0</v>
       </c>
       <c r="E3" s="3" t="n">
+        <v>22.0</v>
+      </c>
+    </row>
+    <row r="4" ht="54.0" customHeight="true">
+      <c r="A4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>260.0</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>225.0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>24.0</v>
+      </c>
+    </row>
+    <row r="5" ht="54.0" customHeight="true">
+      <c r="A5" s="4" t="n">
+        <v>170.0</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>290.0</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>230.0</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>250.0</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>26.0</v>
+      </c>
+    </row>
+    <row r="6" ht="54.0" customHeight="true">
+      <c r="A6" s="5" t="n">
+        <v>190.0</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>325.0</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>260.0</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>275.0</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>28.0</v>
+      </c>
+    </row>
+    <row r="7" ht="54.0" customHeight="true">
+      <c r="A7" s="4" t="n">
+        <v>215.0</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>360.0</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>290.0</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>300.0</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>30.0</v>
+      </c>
+    </row>
+    <row r="8" ht="54.0" customHeight="true">
+      <c r="A8" s="5" t="n">
+        <v>240.0</v>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>395.0</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>320.0</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>325.0</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>32.0</v>
+      </c>
+    </row>
+    <row r="9" ht="54.0" customHeight="true">
+      <c r="A9" s="4" t="n">
+        <v>265.0</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>430.0</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>350.0</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>350.0</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>34.0</v>
+      </c>
+    </row>
+    <row r="10" ht="54.0" customHeight="true">
+      <c r="A10" s="5" t="n">
+        <v>290.0</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>465.0</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>380.0</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>375.0</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>36.0</v>
+      </c>
+    </row>
+    <row r="11" ht="54.0" customHeight="true">
+      <c r="A11" s="4" t="n">
+        <v>315.0</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>500.0</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>410.0</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>400.0</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>38.0</v>
+      </c>
+    </row>
+    <row r="12" ht="54.0" customHeight="true">
+      <c r="A12" s="5" t="n">
+        <v>340.0</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>535.0</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>440.0</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>425.0</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>40.0</v>
+      </c>
+    </row>
+    <row r="13" ht="54.0" customHeight="true">
+      <c r="A13" s="4" t="n">
+        <v>380.0</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>585.0</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>485.0</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>465.0</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>42.0</v>
+      </c>
+    </row>
+    <row r="14" ht="54.0" customHeight="true">
+      <c r="A14" s="5" t="n">
+        <v>405.0</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>620.0</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>535.0</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>490.0</v>
+      </c>
+      <c r="E14" s="3" t="n">
         <v>44.0</v>
       </c>
     </row>
-    <row r="4" ht="54.0" customHeight="true">
-      <c r="A4" s="7" t="n">
-        <v>400.0</v>
-      </c>
-      <c r="B4" s="7" t="n">
-        <v>625.0</v>
-      </c>
-      <c r="C4" s="7" t="n">
+    <row r="15" ht="54.0" customHeight="true">
+      <c r="A15" s="4" t="n">
+        <v>435.0</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>660.0</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>585.0</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>515.0</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>46.0</v>
+      </c>
+    </row>
+    <row r="16" ht="54.0" customHeight="true">
+      <c r="A16" s="5" t="n">
+        <v>470.0</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>715.0</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>635.0</v>
+      </c>
+      <c r="D16" s="5" t="n">
         <v>555.0</v>
       </c>
-      <c r="D4" s="7" t="n">
-        <v>480.0</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>46.0</v>
-      </c>
-    </row>
-    <row r="5" ht="54.0" customHeight="true">
-      <c r="A5" s="6" t="n">
-        <v>435.0</v>
-      </c>
-      <c r="B5" s="6" t="n">
-        <v>675.0</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>605.0</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>520.0</v>
-      </c>
-      <c r="E5" s="3" t="n">
+      <c r="E16" s="3" t="n">
         <v>48.0</v>
       </c>
     </row>
-    <row r="6" ht="54.0" customHeight="true">
-      <c r="A6" s="7" t="n">
-        <v>475.0</v>
-      </c>
-      <c r="B6" s="7" t="n">
-        <v>730.0</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>655.0</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>560.0</v>
-      </c>
-      <c r="E6" s="3" t="n">
+    <row r="17" ht="54.0" customHeight="true">
+      <c r="A17" s="4" t="n">
+        <v>510.0</v>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>770.0</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>685.0</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>595.0</v>
+      </c>
+      <c r="E17" s="3" t="n">
         <v>50.0</v>
       </c>
     </row>
-    <row r="7" ht="54.0" customHeight="true">
-      <c r="A7" s="6" t="n">
-        <v>515.0</v>
-      </c>
-      <c r="B7" s="6" t="n">
+    <row r="18" ht="54.0" customHeight="true">
+      <c r="A18" s="5" t="n">
+        <v>550.0</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>825.0</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>735.0</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>635.0</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>52.0</v>
+      </c>
+    </row>
+    <row r="19" ht="54.0" customHeight="true">
+      <c r="A19" s="4" t="n">
+        <v>590.0</v>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>880.0</v>
+      </c>
+      <c r="C19" s="4" t="n">
         <v>785.0</v>
       </c>
-      <c r="C7" s="6" t="n">
-        <v>705.0</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>605.0</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>52.0</v>
-      </c>
-    </row>
-    <row r="8" ht="54.0" customHeight="true">
-      <c r="A8" s="7" t="n">
-        <v>555.0</v>
-      </c>
-      <c r="B8" s="7" t="n">
-        <v>845.0</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>755.0</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>650.0</v>
-      </c>
-      <c r="E8" s="3" t="n">
+      <c r="D19" s="4" t="n">
+        <v>680.0</v>
+      </c>
+      <c r="E19" s="3" t="n">
         <v>54.0</v>
       </c>
     </row>
-    <row r="9" ht="54.0" customHeight="true">
-      <c r="A9" s="6" t="n">
-        <v>595.0</v>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>905.0</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>805.0</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>695.0</v>
-      </c>
-      <c r="E9" s="3" t="n">
+    <row r="20" ht="54.0" customHeight="true">
+      <c r="A20" s="5" t="n">
+        <v>630.0</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>935.0</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>835.0</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>725.0</v>
+      </c>
+      <c r="E20" s="3" t="n">
         <v>56.0</v>
       </c>
     </row>

</xml_diff>